<commit_message>
feat(compensation): HCM_10 Phase C — merit matrix + budgets (M363-M364)
M363: merit_matrix + cells (V202, DEFAULT seeded with PRD §11 grid 4 bands×3
positions). suggest(employeeId) maps latest performance finalRating->band
(>=4.5 EXC / >=3.5 GOOD / >=2.5 MEETS / else BELOW) and range penetration->
LOW/MID/HIGH, returns merit% + amount + new salary. SPA editable grid + suggest panel.
M364: compensation_budget (scope GLOBAL/DEPT/MANAGER/GRADE/LEGAL_ENTITY, type
MERIT/BONUS/INCENTIVE/PROMOTION, amount/consumed/remaining). Wired into salary-change
create (HARD_STOP blocks, EXCEPTION_APPROVAL raises OVER_BUDGET, WARNING proceeds) and
consumes on apply. SPA budgets page with consumed/remaining bars.

Boot-verified: V202 applied, 12 merit cells seeded, JPA validate OK, started 33s.
SPA build clean. UAT Excel -> 37 cases (A16 + B13 + C8).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
+++ b/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1526,9 +1526,241 @@
       <c r="F30" s="8" t="inlineStr"/>
       <c r="G30" s="7" t="inlineStr"/>
     </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>MM-01</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Merit Matrix (M363)</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Compensation → Merit Matrices → open the DEFAULT matrix.</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>A grid shows 4 performance bands (Excellent/Good/Meets/Below) × 3 range positions (Low/Mid/High) with the seeded percentages: Excellent 8/6/4, Good 5/4/2, Meets 3/2/1, Below 0/0/0.</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr"/>
+      <c r="G31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>MM-02</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Merit Matrix (M363)</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Change one cell (e.g. Good/Mid from 4 to 4.5) and Save.</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>The change is saved and shows the new value when reopened.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>MM-03</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Merit Matrix (M363)</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Use the 'Suggest merit' panel: pick the test employee.</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>It shows the employee's performance band, range position, suggested merit %, current salary, merit amount and new salary. Check: merit amount = current salary × merit % ÷ 100, and new salary = current + merit amount.</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr"/>
+      <c r="G33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34" ht="57" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>BUD-01</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Budgets (M364)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Compensation → Budgets → Create. Budget Type=MERIT, Scope=GLOBAL, Amount=10000, Currency=AZN, Effective From=today. Save.</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>The budget appears with Amount 10000, Consumed 0, Remaining 10000.</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>BUD-02</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Budgets (M364)</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>With Settings → Budget policy = WARNING, create a salary change whose increase is larger than the remaining budget.</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>The salary change is still allowed (WARNING policy only warns, does not block).</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr"/>
+      <c r="G35" s="10" t="inlineStr"/>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>BUD-03</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Budgets (M364)</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>In Settings set Budget policy = HARD_STOP. Create a salary change whose increase exceeds the remaining MERIT budget.</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>The salary change is blocked with a 'budget exceeded' error.</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr"/>
+      <c r="G36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37" ht="57" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>BUD-04</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Budgets (M364)</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>Set Budget policy back to WARNING. Approve a salary change (via the Approvals inbox) for a budgeted employee, then reopen the MERIT budget.</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>The budget's Consumed has increased by the salary increase and Remaining has decreased accordingly.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr"/>
+      <c r="G37" s="10" t="inlineStr"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>BUD-05</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Budgets (M364)</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>On a budget row click Deactivate.</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>The budget shows Inactive (not physically deleted).</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1542,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E16"/>
+  <dimension ref="B1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1644,30 +1876,50 @@
     <row r="10">
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>Merit Matrix (MM)</t>
         </is>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="15" t="n"/>
       <c r="E10" s="15" t="n"/>
     </row>
-    <row r="13">
-      <c r="B13" s="16" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Budgets (BUD)</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Phase A decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="17" t="inlineStr">
+      <c r="C15" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Tester name:</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="17" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="17" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
@@ -1675,7 +1927,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(compensation): HCM_10 Phase D — incentive + commission plans (M365-M366)
M365: incentive_plan + incentive_payout (V203). Payout curve: <threshold(80) 0;
threshold->target linear to target_pct; target->cap linear to max_payout_pct; >cap
capped. amount = eligible_salary x payout_pct. M366: commission_plan + tiers +
commission_payout; flat or marginal-tiered commission on a (stub) sales input.
Both payouts: create(DRAFT) -> approve(APPROVED) -> cancel(DRAFT only).

FIX (caught pre-runtime): approve() no longer creates a payroll_bonus with run_id=NULL
(payroll_bonus.run_id is NOT NULL — would have thrown on first approval). Approval now
only marks APPROVED; the controlled comp->payroll transfer (M369, Phase E) resolves the
target run and pushes approved one-time comp idempotently.

Boot-verified: V203 applied, JPA validate OK, started 30s. SPA build clean.
UAT Excel -> 46 cases (A16 + B13 + C8 + D9).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
+++ b/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1758,9 +1758,270 @@
       <c r="F38" s="8" t="inlineStr"/>
       <c r="G38" s="7" t="inlineStr"/>
     </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>IN-01</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Incentives (M365)</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Compensation → Incentives → Plans tab → Create. Code=SALES_INC, Name=Sales Incentive, Measure=SALES, Target %=10, Threshold achievement=80, Target achievement=100, Cap achievement=120, Max payout %=15. Save.</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>The incentive plan appears in the Plans table.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr"/>
+      <c r="G39" s="10" t="inlineStr"/>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>IN-02</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Incentives (M365)</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Payouts tab → New payout. Pick the plan + test employee, Period=2026-Q1, Achievement %=100. Save.</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Payout is created with payout amount = eligible salary × 10% (the target). E.g. salary 2500 → payout 250.</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>IN-03</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Incentives (M365)</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Create another payout with Achievement %=70 (below the 80 threshold).</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Payout amount is 0 (below threshold = no payout).</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr"/>
+      <c r="G41" s="10" t="inlineStr"/>
+    </row>
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>IN-04</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Incentives (M365)</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Create a payout with Achievement %=120 (at the cap).</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Payout uses the maximum payout % (capped); e.g. salary 2500 × 15% = 375.</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43" ht="42" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>IN-05</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Incentives (M365)</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>On a DRAFT payout click Approve.</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="inlineStr">
+        <is>
+          <t>Status becomes APPROVED. A note explains it is not attached to payroll until the Payroll-transfer step (Phase E).</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr"/>
+      <c r="G43" s="10" t="inlineStr"/>
+    </row>
+    <row r="44" ht="57" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>CM-01</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Commission (M366)</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Compensation → Commission → Plans → Create. Code=REV_2PCT, Name=Revenue 2%, Basis=REVENUE, Tiered=off, Flat rate %=2. Save.</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>The commission plan appears.</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr"/>
+      <c r="G44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45" ht="42" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>CM-02</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Commission (M366)</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>Payouts tab → New payout. Pick the plan + employee, Period=2026-01, Sales amount=10000. Save.</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="inlineStr">
+        <is>
+          <t>Commission amount = 200 (2% of 10000).</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr"/>
+      <c r="G45" s="10" t="inlineStr"/>
+    </row>
+    <row r="46" ht="42" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>CM-03</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Commission (M366)</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Create a tiered plan (Tiered=on) with tiers e.g. 0–5000 @1%, 5000+ @3%. Create a payout with Sales amount=10000.</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Commission uses marginal tiers: 5000×1% + 5000×3% = 50 + 150 = 200.</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr"/>
+    </row>
+    <row r="47" ht="42" customHeight="1">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>CM-04</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Commission (M366)</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>On a DRAFT commission payout click Approve.</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>Status becomes APPROVED (attached to payroll later via the Payroll-transfer step).</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr"/>
+      <c r="G47" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1774,7 +2035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E18"/>
+  <dimension ref="B1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1896,30 +2157,50 @@
     <row r="12">
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>Incentives (IN)</t>
         </is>
       </c>
       <c r="C12" s="14" t="n"/>
       <c r="D12" s="15" t="n"/>
       <c r="E12" s="15" t="n"/>
     </row>
-    <row r="15">
-      <c r="B15" s="16" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Commission (CM)</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Phase A decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="17" t="inlineStr">
+      <c r="C17" s="14" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Tester name:</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="17" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
@@ -1927,7 +2208,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(compensation): HCM_10 Phase E — market data, total-comp statement, payroll transfer (M367-M369)
M367: market_salary_survey + market_salary_data (percentiles) + compare(employee)
-> market ratio = salary/p50x100. M368: total_comp_statement = base + allowances +
bonus + incentives + commission + employer contributions (from payroll_result
employer DSMF/MMI/unemployment); PDF via PayslipPdfService pattern -> MinIO;
generate/release + employee self-service download of own RELEASED statement.
M369: payroll_comp_transfer — the controlled bridge that pushes APPROVED incentive/
commission payouts to a chosen OPEN payroll run via PayrollRunService.addBonus
(real run_id), idempotent (UNIQUE source + payroll_bonus_id guard), skips terminated;
payout -> PAID.

Boot-verified: V204 applied, JPA validate OK, endpoints secured (401), started 36s.
SPA build clean. UAT Excel -> 54 cases (A16 B13 C8 D9 E8).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
+++ b/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2019,9 +2019,241 @@
       <c r="F47" s="8" t="inlineStr"/>
       <c r="G47" s="10" t="inlineStr"/>
     </row>
+    <row r="48" ht="72" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>MK-01</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Market Data (M367)</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Compensation → Market Data → create a survey (Provider=Mercer, Year=2026). Select it → add a data row (Grade code = the test grade, p25=1800, p50=2400, p75=3000, p90=3600). Then use 'Compare employee' → pick the test employee.</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>The comparison shows the percentiles, the employee salary, the market ratio (salary ÷ p50 × 100) and a position label (below/at/above market).</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr"/>
+    </row>
+    <row r="49" ht="57" customHeight="1">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>TC-01</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Total Comp (M368)</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Compensation → Total Comp Statements → pick the year → Generate all.</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>A statement per employee appears with base + allowances + bonus + incentives + commission + employer contributions, and a Total that equals the sum of those parts.</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr"/>
+      <c r="G49" s="10" t="inlineStr"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>TC-02</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Total Comp (M368)</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>On a GENERATED statement click Release (or Release all).</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Status changes to RELEASED.</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr"/>
+    </row>
+    <row r="51" ht="42" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Total Comp (M368)</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Click Download on a statement.</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>A PDF opens showing the compensation breakdown and the total.</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr"/>
+      <c r="G51" s="10" t="inlineStr"/>
+    </row>
+    <row r="52" ht="42" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Total Comp (M368)</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Sign in as the Employee → My Workspace → Payroll tab → My total compensation → pick the year → Download.</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>The employee can download their own RELEASED total-compensation statement only.</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
+    </row>
+    <row r="53" ht="72" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>TR-01</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Payroll Transfer (M369)</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Compensation → Payroll Transfer. Select an OPEN payroll run (not Paid) and click 'Transfer approved payouts to this run'.</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>A result shows how many were transferred; the previously-approved incentive/commission payouts become PAID and appear as one-time bonuses on that payroll run; a transfer-log row is recorded.</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr"/>
+      <c r="G53" s="10" t="inlineStr"/>
+    </row>
+    <row r="54" ht="42" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>TR-02</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Payroll Transfer (M369)</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Click Transfer again for the SAME run.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>0 payouts are transferred the second time (idempotent — no duplicates).</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr"/>
+    </row>
+    <row r="55" ht="42" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>TR-03</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Payroll Transfer (M369)</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Approve a payout for a TERMINATED employee, then run the transfer.</t>
+        </is>
+      </c>
+      <c r="E55" s="10" t="inlineStr">
+        <is>
+          <t>That payout is skipped (terminated employees are not transferred to payroll).</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr"/>
+      <c r="G55" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2035,7 +2267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E20"/>
+  <dimension ref="B1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2177,30 +2409,60 @@
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>Market Data (MK)</t>
         </is>
       </c>
       <c r="C14" s="14" t="n"/>
       <c r="D14" s="15" t="n"/>
       <c r="E14" s="15" t="n"/>
     </row>
+    <row r="15">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Total Comp (TC)</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Payroll Transfer (TR)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+    </row>
     <row r="17">
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Phase A decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="17" t="inlineStr">
+      <c r="C20" s="14" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Tester name:</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="17" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
@@ -2208,7 +2470,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(compensation): HCM_10 Phase F — dashboard, analytics, comp letters, notifications (M370-M371)
M370: CompensationDashboardService (read-only, scope-aware) — headcount/without-grade/
without-band/out-of-band, pending approvals, open exceptions, compa-ratio distribution
(reuses CompRatioService buckets), budget utilization; + reports (compa-ratio dist,
out-of-band, budget-vs-actual). SPA dashboard (Recharts) as the Compensation landing.
M371: salary-increase letter via the reused letter engine (V205 seeds SALARY_INCREASE_
LETTER template en+az) — generated for APPLIED changes; 'Generate Letter' action on the
Salary Changes page. Notifications: reused NotificationService.notifyAll on salary-change
submit (manager), approval (employee), and exception raised (manager) — non-fatal.

Boot-verified: V205 applied, JPA validate OK, Started HcmApplication, dashboard beans
wired. SPA build clean. UAT Excel -> 62 cases (all 6 phases A–F).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
+++ b/PRD/HCM_10_Compensation_Management_Multi_Tenant_PRD/Compensation_UAT_Test_Script.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Phase A — Pay Bands, Settings, Change Reasons, Compensation Profile (compa-ratio + range penetration + history). Phase B — Salary-change requests with approval-before-payroll (a change only becomes the employee's salary after it is approved) + auto-raised Compensation Exceptions (out-of-band / above-threshold). Later phases (merit cycles, budgets, incentives/commission, market data, total-comp statement, payroll transfer) will be appended to this same file.</t>
+          <t>Phases A–F COMPLETE — Pay Bands, Settings, Change Reasons, Compensation Profile; Salary-change approvals + Exceptions; Merit Matrix + Budgets; Incentives + Commission; Market Data + Total-Comp Statement + Payroll Transfer; Dashboard/Analytics + Comp Letters + Notifications. The whole Compensation module is covered here.</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2251,9 +2251,241 @@
       <c r="F55" s="8" t="inlineStr"/>
       <c r="G55" s="10" t="inlineStr"/>
     </row>
+    <row r="56" ht="57" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>DB-01</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard (M370)</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Compensation → Dashboard.</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Stat cards populate: employees with a comp record, without grade, without band, out of band, pending salary-change approvals, and open exceptions — with sensible numbers.</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr"/>
+    </row>
+    <row r="57" ht="42" customHeight="1">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>DB-02</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard (M370)</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Look at the Compa-ratio distribution chart.</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>A bar chart shows counts across bands (below-min / low / mid / high / above-max), colour-coded.</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr"/>
+      <c r="G57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58" ht="42" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>DB-03</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard (M370)</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Look at the Budget utilization table.</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Each active budget shows amount, consumed, remaining and a utilization % progress bar.</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59" ht="42" customHeight="1">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>DB-04</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>Dashboard (M370)</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>Look at the Out-of-band employees table (also under Reports).</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>It lists employees whose salary is outside their pay band, with the delta.</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr"/>
+      <c r="G59" s="10" t="inlineStr"/>
+    </row>
+    <row r="60" ht="42" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>DB-05</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Dashboard (M370)</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Department Manager</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>Sign in as a Department Manager and open the Dashboard.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>The figures reflect only your team (hierarchy-scoped), not the whole company.</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr"/>
+      <c r="G60" s="7" t="inlineStr"/>
+    </row>
+    <row r="61" ht="42" customHeight="1">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>LT-01</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>Comp Letters (M371)</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>On Salary Changes, find an APPLIED change and click 'Generate Letter'.</t>
+        </is>
+      </c>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>A salary-increase letter PDF opens showing employee name, old salary, new salary, increase % and effective date.</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr"/>
+      <c r="G61" s="10" t="inlineStr"/>
+    </row>
+    <row r="62" ht="42" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>LT-02</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Comp Letters (M371)</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>HR Admin</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Look at the 'Generate Letter' action on a DRAFT / PENDING change.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>It is disabled — a letter is only available once the change is APPLIED.</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr"/>
+      <c r="G62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63" ht="57" customHeight="1">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>NT-01</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Notifications (M371)</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>Manager / Employee</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>Submit a salary change (manager is notified), approve it (employee is notified), and trigger an exception (HR/manager notified). Check the notifications bell.</t>
+        </is>
+      </c>
+      <c r="E63" s="10" t="inlineStr">
+        <is>
+          <t>The relevant users receive in-app notifications for submit / approval / exception events.</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr"/>
+      <c r="G63" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2267,7 +2499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E23"/>
+  <dimension ref="B1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2439,38 +2671,48 @@
     <row r="17">
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Permissions (SEC)</t>
+          <t>Dashboard + Letters (DB/LT/NT)</t>
         </is>
       </c>
       <c r="C17" s="14" t="n"/>
       <c r="D17" s="15" t="n"/>
       <c r="E17" s="15" t="n"/>
     </row>
-    <row r="20">
-      <c r="B20" s="16" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Permissions (SEC)</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Phase A decision (SHIP / DON'T SHIP):</t>
         </is>
       </c>
-      <c r="C20" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>Tester name:</t>
-        </is>
-      </c>
+      <c r="C21" s="14" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="17" t="inlineStr">
         <is>
+          <t>Tester name:</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="17" t="inlineStr">
+        <is>
           <t>Date:</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>